<commit_message>
Feat: File parsing test, change the example
</commit_message>
<xml_diff>
--- a/public/examples/courses_example.xlsx
+++ b/public/examples/courses_example.xlsx
@@ -397,25 +397,41 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:AG6"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="4" width="35.83203125" customWidth="1"/>
     <col min="5" max="5" width="8.83203125" customWidth="1"/>
-    <col min="6" max="6" width="35.83203125" customWidth="1"/>
-    <col min="7" max="7" width="8.83203125" customWidth="1"/>
-    <col min="8" max="8" width="60.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="35.83203125" customWidth="1"/>
+    <col min="8" max="8" width="8.83203125" customWidth="1"/>
     <col min="9" max="9" width="60.83203125" customWidth="1"/>
-    <col min="10" max="10" width="20.83203125" customWidth="1"/>
-    <col min="11" max="11" width="60.83203125" customWidth="1"/>
-    <col min="12" max="12" width="20.83203125" customWidth="1"/>
-    <col min="13" max="13" width="40.83203125" customWidth="1"/>
+    <col min="10" max="10" width="60.83203125" customWidth="1"/>
+    <col min="11" max="11" width="20.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1"/>
+    <col min="13" max="13" width="20.83203125" customWidth="1"/>
     <col min="14" max="14" width="40.83203125" customWidth="1"/>
-    <col min="15" max="15" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="40.83203125" customWidth="1"/>
     <col min="16" max="16" width="12.83203125" customWidth="1"/>
     <col min="17" max="17" width="12.83203125" customWidth="1"/>
+    <col min="18" max="18" width="14.83203125" customWidth="1"/>
+    <col min="19" max="19" width="14.83203125" customWidth="1"/>
+    <col min="20" max="20" width="12.83203125" customWidth="1"/>
+    <col min="21" max="21" width="12.83203125" customWidth="1"/>
+    <col min="22" max="22" width="12.83203125" customWidth="1"/>
+    <col min="23" max="23" width="12.83203125" customWidth="1"/>
+    <col min="24" max="24" width="12.83203125" customWidth="1"/>
+    <col min="25" max="25" width="12.83203125" customWidth="1"/>
+    <col min="26" max="26" width="12.83203125" customWidth="1"/>
+    <col min="27" max="27" width="12.83203125" customWidth="1"/>
+    <col min="28" max="28" width="12.83203125" customWidth="1"/>
+    <col min="29" max="29" width="12.83203125" customWidth="1"/>
+    <col min="30" max="30" width="12.83203125" customWidth="1"/>
+    <col min="31" max="31" width="12.83203125" customWidth="1"/>
+    <col min="32" max="32" width="12.83203125" customWidth="1"/>
+    <col min="33" max="33" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -435,40 +451,88 @@
         <v>code</v>
       </c>
       <c r="F1" t="str">
+        <v>id</v>
+      </c>
+      <c r="G1" t="str">
         <v>name</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>credits</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>learning_outcomes</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>content</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>instructor</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>description</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>prerequisites</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>assessment</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>url</v>
       </c>
-      <c r="O1" t="str">
-        <v>1ST_YEAR_1P</v>
-      </c>
       <c r="P1" t="str">
-        <v>1ST_YEAR_2P</v>
+        <v>start_date</v>
       </c>
       <c r="Q1" t="str">
-        <v>2ND_YEAR_1P</v>
+        <v>end_date</v>
+      </c>
+      <c r="R1" t="str">
+        <v>enrollment_start_date</v>
+      </c>
+      <c r="S1" t="str">
+        <v>enrollment_end_date</v>
+      </c>
+      <c r="T1" t="str">
+        <v>1st_YEAR_1P</v>
+      </c>
+      <c r="U1" t="str">
+        <v>1st_YEAR_2P</v>
+      </c>
+      <c r="V1" t="str">
+        <v>1st_YEAR_3P</v>
+      </c>
+      <c r="W1" t="str">
+        <v>1st_YEAR_4P</v>
+      </c>
+      <c r="X1" t="str">
+        <v>1st_YEAR_5P</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>2nd_YEAR_1P</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>2nd_YEAR_2P</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>2nd_YEAR_3P</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>2nd_YEAR_4P</v>
+      </c>
+      <c r="AC1" t="str">
+        <v>2nd_YEAR_5P</v>
+      </c>
+      <c r="AD1" t="str">
+        <v>3rd_YEAR_1P</v>
+      </c>
+      <c r="AE1" t="str">
+        <v>3rd_YEAR_2P</v>
+      </c>
+      <c r="AF1" t="str">
+        <v>3rd_YEAR_3P</v>
+      </c>
+      <c r="AG1" t="str">
+        <v>3rd_YEAR_4P</v>
       </c>
     </row>
     <row r="2">
@@ -488,40 +552,88 @@
         <v>CS101</v>
       </c>
       <c r="F2" t="str">
+        <v>1001</v>
+      </c>
+      <c r="G2" t="str">
         <v>Introduction to Programming</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>6</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>Understand fundamental programming concepts; Write clean and readable code; Debug and test simple programs; Apply problem-solving strategies</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>Variables and data types; Control flow (if/else, loops); Functions and scope; Introduction to arrays and strings; Basic file I/O</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v>Dr. Alice Nguyen</v>
       </c>
-      <c r="K2" t="str">
-        <v>A foundational course covering core programming concepts using Python. Students will build small projects from the ground up.</v>
-      </c>
       <c r="L2" t="str">
         <v/>
       </c>
       <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
         <v>Written exam 40%; Programming assignments 40%; Lab participation 20%</v>
       </c>
-      <c r="N2" t="str">
+      <c r="O2" t="str">
         <v>https://university.edu/courses/cs101</v>
       </c>
-      <c r="O2">
-        <v>1</v>
-      </c>
-      <c r="P2">
-        <v>1</v>
-      </c>
-      <c r="Q2">
-        <v>0</v>
+      <c r="P2" t="str">
+        <v>2026-09-01</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>2026-12-15</v>
+      </c>
+      <c r="R2" t="str">
+        <v>2026-06-01</v>
+      </c>
+      <c r="S2" t="str">
+        <v>2026-08-25</v>
+      </c>
+      <c r="T2" t="str">
+        <v>x</v>
+      </c>
+      <c r="U2" t="str">
+        <v>x</v>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
+        <v/>
+      </c>
+      <c r="Z2" t="str">
+        <v/>
+      </c>
+      <c r="AA2" t="str">
+        <v/>
+      </c>
+      <c r="AB2" t="str">
+        <v/>
+      </c>
+      <c r="AC2" t="str">
+        <v/>
+      </c>
+      <c r="AD2" t="str">
+        <v/>
+      </c>
+      <c r="AE2" t="str">
+        <v/>
+      </c>
+      <c r="AF2" t="str">
+        <v/>
+      </c>
+      <c r="AG2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -541,40 +653,88 @@
         <v>CS201</v>
       </c>
       <c r="F3" t="str">
+        <v>1002</v>
+      </c>
+      <c r="G3" t="str">
         <v>Data Structures and Algorithms</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>6</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>Implement common data structures; Analyse algorithm time and space complexity; Choose appropriate data structures for a given problem</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <v>Linked lists; Stacks and queues; Trees and graphs; Sorting and searching algorithms; Big-O notation</v>
       </c>
-      <c r="J3" t="str">
+      <c r="K3" t="str">
         <v>Prof. John Smith</v>
       </c>
-      <c r="K3" t="str">
-        <v>Covers the design and analysis of fundamental data structures and algorithms. Prerequisite for most upper-level CS courses.</v>
-      </c>
       <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
         <v>CS101</v>
       </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
         <v>Written exam 50%; Programming assignments 35%; Quizzes 15%</v>
       </c>
-      <c r="N3" t="str">
+      <c r="O3" t="str">
         <v>https://university.edu/courses/cs201</v>
       </c>
-      <c r="O3">
-        <v>0</v>
-      </c>
-      <c r="P3">
-        <v>0</v>
-      </c>
-      <c r="Q3">
-        <v>1</v>
+      <c r="P3" t="str">
+        <v>2027-01-10</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>2027-03-20</v>
+      </c>
+      <c r="R3" t="str">
+        <v>2026-11-01</v>
+      </c>
+      <c r="S3" t="str">
+        <v>2027-01-05</v>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v/>
+      </c>
+      <c r="X3" t="str">
+        <v/>
+      </c>
+      <c r="Y3" t="str">
+        <v>x</v>
+      </c>
+      <c r="Z3" t="str">
+        <v/>
+      </c>
+      <c r="AA3" t="str">
+        <v/>
+      </c>
+      <c r="AB3" t="str">
+        <v/>
+      </c>
+      <c r="AC3" t="str">
+        <v/>
+      </c>
+      <c r="AD3" t="str">
+        <v/>
+      </c>
+      <c r="AE3" t="str">
+        <v/>
+      </c>
+      <c r="AF3" t="str">
+        <v/>
+      </c>
+      <c r="AG3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -594,40 +754,88 @@
         <v>CS301</v>
       </c>
       <c r="F4" t="str">
+        <v>1003</v>
+      </c>
+      <c r="G4" t="str">
         <v>Database Systems</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>5</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>Design relational schemas; Write complex SQL queries; Understand transaction management; Apply normalisation techniques</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>Entity-Relationship modelling; SQL (DDL &amp; DML); Joins and subqueries; Normalisation (1NF-3NF); Indexing and query optimisation; Transactions and ACID properties</v>
       </c>
-      <c r="J4" t="str">
+      <c r="K4" t="str">
         <v>Dr. Maria Santos</v>
       </c>
-      <c r="K4" t="str">
-        <v>An introduction to relational database theory and practice. Students will design schemas and implement full database applications.</v>
-      </c>
       <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
         <v>CS201</v>
       </c>
-      <c r="M4" t="str">
+      <c r="N4" t="str">
         <v>Project 40%; Midterm exam 30%; Weekly SQL exercises 30%</v>
       </c>
-      <c r="N4" t="str">
+      <c r="O4" t="str">
         <v>https://university.edu/courses/cs301</v>
       </c>
-      <c r="O4">
-        <v>0</v>
-      </c>
-      <c r="P4">
-        <v>0</v>
-      </c>
-      <c r="Q4">
-        <v>1</v>
+      <c r="P4" t="str">
+        <v>2027-01-10</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>2027-03-20</v>
+      </c>
+      <c r="R4" t="str">
+        <v>2026-11-01</v>
+      </c>
+      <c r="S4" t="str">
+        <v>2027-01-05</v>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
+        <v/>
+      </c>
+      <c r="Y4" t="str">
+        <v/>
+      </c>
+      <c r="Z4" t="str">
+        <v>x</v>
+      </c>
+      <c r="AA4" t="str">
+        <v/>
+      </c>
+      <c r="AB4" t="str">
+        <v/>
+      </c>
+      <c r="AC4" t="str">
+        <v/>
+      </c>
+      <c r="AD4" t="str">
+        <v/>
+      </c>
+      <c r="AE4" t="str">
+        <v/>
+      </c>
+      <c r="AF4" t="str">
+        <v/>
+      </c>
+      <c r="AG4" t="str">
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -647,40 +855,88 @@
         <v>CS402</v>
       </c>
       <c r="F5" t="str">
+        <v>1004</v>
+      </c>
+      <c r="G5" t="str">
         <v>Cloud Computing Fundamentals</v>
       </c>
-      <c r="G5" t="str">
+      <c r="H5" t="str">
         <v>5</v>
       </c>
-      <c r="H5" t="str">
+      <c r="I5" t="str">
         <v>Deploy applications on cloud platforms; Configure virtual machines and storage; Apply cloud security best practices</v>
       </c>
-      <c r="I5" t="str">
+      <c r="J5" t="str">
         <v>Cloud service models (IaaS, PaaS, SaaS); AWS and Azure basics; Containerisation with Docker; Serverless architectures; Cloud cost management</v>
       </c>
-      <c r="J5" t="str">
+      <c r="K5" t="str">
         <v>Dr. Kevin Lee</v>
       </c>
-      <c r="K5" t="str">
-        <v>Introduces cloud computing concepts and hands-on practice with major cloud providers. Focus on practical deployment skills.</v>
-      </c>
       <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
         <v>CS301</v>
       </c>
-      <c r="M5" t="str">
+      <c r="N5" t="str">
         <v>Cloud project 50%; Presentations 20%; Online quizzes 30%</v>
       </c>
-      <c r="N5" t="str">
+      <c r="O5" t="str">
         <v>https://university.edu/courses/cs402</v>
       </c>
-      <c r="O5">
-        <v>0</v>
-      </c>
-      <c r="P5">
-        <v>0</v>
-      </c>
-      <c r="Q5">
-        <v>0</v>
+      <c r="P5" t="str">
+        <v>2027-03-21</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>2027-05-30</v>
+      </c>
+      <c r="R5" t="str">
+        <v>2027-01-06</v>
+      </c>
+      <c r="S5" t="str">
+        <v>2027-03-15</v>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
+      <c r="W5" t="str">
+        <v/>
+      </c>
+      <c r="X5" t="str">
+        <v/>
+      </c>
+      <c r="Y5" t="str">
+        <v/>
+      </c>
+      <c r="Z5" t="str">
+        <v/>
+      </c>
+      <c r="AA5" t="str">
+        <v>x</v>
+      </c>
+      <c r="AB5" t="str">
+        <v/>
+      </c>
+      <c r="AC5" t="str">
+        <v/>
+      </c>
+      <c r="AD5" t="str">
+        <v/>
+      </c>
+      <c r="AE5" t="str">
+        <v/>
+      </c>
+      <c r="AF5" t="str">
+        <v/>
+      </c>
+      <c r="AG5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -700,45 +956,93 @@
         <v>AI501</v>
       </c>
       <c r="F6" t="str">
+        <v>1005</v>
+      </c>
+      <c r="G6" t="str">
         <v>Machine Learning</v>
       </c>
-      <c r="G6" t="str">
+      <c r="H6" t="str">
         <v>7</v>
       </c>
-      <c r="H6" t="str">
+      <c r="I6" t="str">
         <v>Build and evaluate supervised and unsupervised models; Apply feature engineering techniques; Interpret model outputs</v>
       </c>
-      <c r="I6" t="str">
+      <c r="J6" t="str">
         <v>Linear and logistic regression; Decision trees and random forests; Neural networks; Model evaluation metrics; Cross-validation; Bias-variance tradeoff</v>
       </c>
-      <c r="J6" t="str">
+      <c r="K6" t="str">
         <v>Prof. Sarah Kim</v>
       </c>
-      <c r="K6" t="str">
-        <v>A graduate-level treatment of machine learning theory and application. Students implement models from scratch and via scikit-learn.</v>
-      </c>
       <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
         <v>CS201</v>
       </c>
-      <c r="M6" t="str">
+      <c r="N6" t="str">
         <v>Research paper 30%; Implementation projects 40%; Final exam 30%</v>
       </c>
-      <c r="N6" t="str">
+      <c r="O6" t="str">
         <v>https://university.edu/courses/ai501</v>
       </c>
-      <c r="O6">
-        <v>0</v>
-      </c>
-      <c r="P6">
-        <v>0</v>
-      </c>
-      <c r="Q6">
-        <v>0</v>
+      <c r="P6" t="str">
+        <v>2026-09-01</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>2026-12-15</v>
+      </c>
+      <c r="R6" t="str">
+        <v>2026-06-01</v>
+      </c>
+      <c r="S6" t="str">
+        <v>2026-08-25</v>
+      </c>
+      <c r="T6" t="str">
+        <v>x</v>
+      </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
+      <c r="V6" t="str">
+        <v/>
+      </c>
+      <c r="W6" t="str">
+        <v/>
+      </c>
+      <c r="X6" t="str">
+        <v/>
+      </c>
+      <c r="Y6" t="str">
+        <v/>
+      </c>
+      <c r="Z6" t="str">
+        <v/>
+      </c>
+      <c r="AA6" t="str">
+        <v/>
+      </c>
+      <c r="AB6" t="str">
+        <v/>
+      </c>
+      <c r="AC6" t="str">
+        <v/>
+      </c>
+      <c r="AD6" t="str">
+        <v/>
+      </c>
+      <c r="AE6" t="str">
+        <v/>
+      </c>
+      <c r="AF6" t="str">
+        <v/>
+      </c>
+      <c r="AG6" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AG6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>